<commit_message>
fix: robust Excel header detection via first-cell match; remove example rows from templates
</commit_message>
<xml_diff>
--- a/datos/interpretation example.xlsx
+++ b/datos/interpretation example.xlsx
@@ -323,7 +323,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="39.13" customWidth="1" style="2" min="1" max="1"/>
@@ -547,130 +547,6 @@
       <c r="U3" s="1" t="n"/>
       <c r="V3" s="1" t="n"/>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Resonancias del Tiempo</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>María López</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2023-04-10</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Festival de Musica Contemporanea</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Auditorio Nacional</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Madrid</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Standard Performance</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Cuarteto Cervantes</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Javier Pérez</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Notas del programa del festival.</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>https://youtu.be/example_live1</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Una experiencia unica interpretar esta obra.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Nocturno para Piano</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Carlos Ruiz</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2022-11-05</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Ciclo Música Nueva</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Sala Gayarre</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Pamplona</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>National Premiere</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Elena Martín (piano)</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Obra de gran delicadeza y precision tecnica.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="C1:D1"/>

</xml_diff>